<commit_message>
feat(demo): batch 3 — first live non-PASS verdicts; workbook now 20 runs
Ten more live Haiku runs: 7 PASS, 2 NEEDS_HUMAN, 1 FAIL — the first
non-PASS verdicts from a live executor, each for an explainable reason:
one wandering CHANGELOG.md edit (review-required path -> escalation),
one CHANGELOG edit plus an incomplete consistency sweep (both modes in
one run), and one clean-looking change that left text-unidecode refs
behind (task-consistency blocking FAIL - the historically most common
blindspot, caught). Combined: 17/20 PASS, 15% observed non-PASS.

Workbook rebuilt: 20 rows, per-row policy hash read from archived
result.json, consistency table computed from archived patches (setup.py
and slugify.py still byte-identical in every run across all batches;
README now at 4/3/5 distinct versions per batch), non-PASS runs
annotated on the summary sheet. Recalc clean.
</commit_message>
<xml_diff>
--- a/demo/runs/sdlc-campaign.xlsx
+++ b/demo/runs/sdlc-campaign.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="123">
   <si>
     <t xml:space="preserve">run_id</t>
   </si>
@@ -152,7 +152,7 @@
     <t xml:space="preserve">2</t>
   </si>
   <si>
-    <t xml:space="preserve">45c94e20</t>
+    <t xml:space="preserve">853db4b4</t>
   </si>
   <si>
     <t xml:space="preserve">sdlc-20260902T193711Z</t>
@@ -182,10 +182,112 @@
     <t xml:space="preserve">2026-09-02 19:41:35</t>
   </si>
   <si>
-    <t xml:space="preserve">SDLC Online Campaign - 10 live runs, gate only, no oracle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Task X1 on python-slugify. Every run: fresh claude -p session (model pinned) edits the repo, release-gate 0.6.0 judges it. No oracle: the verdict IS the outcome, as it would be inside an SDLC. All rows share card sha 9f5ae3e4, base commit 42e5e792, model claude-haiku-4-5-20251001.</t>
+    <t xml:space="preserve">sdlc-20260902T201026Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-02 20:10:26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-20260902T201153Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-02 20:11:53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5494c922c526</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-20260902T201301Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-02 20:13:01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-20260902T201424Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-02 20:14:24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-20260902T201544Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-02 20:15:44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEEDS_HUMAN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSERTION_FAILED;PATH_OUTSIDE_ALLOWED;PATH_REVIEW_REQUIRED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHANGELOG.md|README.md|setup.py|slugify/slugify.py</t>
+  </si>
+  <si>
+    <t xml:space="preserve">66c82cf6110e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-20260902T201654Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-02 20:16:54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-20260902T201815Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-02 20:18:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PATH_OUTSIDE_ALLOWED;PATH_REVIEW_REQUIRED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHANGELOG.md|README.md|setup.py|slugify/slugify.py|tox.ini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">56f934d0c987</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-20260902T201938Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-02 20:19:38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80092727df35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-20260902T202106Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-02 20:21:06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51e4ca76a893</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-20260902T202228Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-02 20:22:28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASSERTION_FAILED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8aee17d64c7a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SDLC Online Campaign - 20 live runs, gate only, no oracle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task X1 on python-slugify. Every run: fresh claude -p session (model pinned, card sha 9f5ae3e4, base 42e5e792) edits the repo; release-gate 0.6.0 judges it. No oracle: the verdict IS the outcome, as inside an SDLC.</t>
   </si>
   <si>
     <t xml:space="preserve">Verdicts</t>
@@ -194,12 +296,6 @@
     <t xml:space="preserve">Averages</t>
   </si>
   <si>
-    <t xml:space="preserve">FAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEEDS_HUMAN</t>
-  </si>
-  <si>
     <t xml:space="preserve">cost / run (USD)</t>
   </si>
   <si>
@@ -212,10 +308,28 @@
     <t xml:space="preserve">output tokens</t>
   </si>
   <si>
-    <t xml:space="preserve">Consistency of changes (the key finding)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All 10 runs changed exactly the same four files: README.md, setup.py, slugify/slugify.py, tox.ini. All 10 whole-diffs are byte-different. Per file, distinct versions produced:</t>
+    <t xml:space="preserve">The three non-PASS runs (batch 3) - each verdict earned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-...201544Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edited CHANGELOG.md (review-required path) AND left the consistency sweep incomplete (task-consistency FAILED). Two failure modes in one run; escalation outranks fail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-...201815Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Did the full task correctly, then also edited CHANGELOG.md - a review-required path. The "wandering edit" escalation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdlc-...202228Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Touched the right 4 files but left text-unidecode references behind: task-consistency ASSERTION_FAILED. The historically most common blindspot, caught as a blocking FAIL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consistency of changes</t>
   </si>
   <si>
     <t xml:space="preserve">file</t>
@@ -227,58 +341,69 @@
     <t xml:space="preserve">batch 2</t>
   </si>
   <si>
+    <t xml:space="preserve">batch 3</t>
+  </si>
+  <si>
     <t xml:space="preserve">reading</t>
   </si>
   <si>
+    <t xml:space="preserve">CHANGELOG.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unrequested edits (2 runs, batch 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">README.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">improvises every time</t>
+  </si>
+  <si>
     <t xml:space="preserve">setup.py</t>
   </si>
   <si>
-    <t xml:space="preserve">IDENTICAL in every run</t>
+    <t xml:space="preserve">byte-identical in every run that touched it</t>
   </si>
   <si>
     <t xml:space="preserve">slugify/slugify.py</t>
   </si>
   <si>
+    <t xml:space="preserve">byte-identical in every run</t>
+  </si>
+  <si>
     <t xml:space="preserve">tox.ini</t>
   </si>
   <si>
     <t xml:space="preserve">minor variants</t>
   </si>
   <si>
-    <t xml:space="preserve">README.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">improvises every time</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stable where it is checked and mechanical (the code); variable where it is prose. Source: per-file patch hashes, computed at batch time (batch-1 patches were later deleted with a workbench rebuild; batch-2 patches archived under demo/runs/sdlc-*-gate/).</t>
+    <t xml:space="preserve">Batch-1 counts are static (its patches were deleted with a workbench rebuild); batches 2-3 computed from archived patches under demo/runs/sdlc-*-gate/.</t>
   </si>
   <si>
     <t xml:space="preserve">Caveats</t>
   </si>
   <si>
-    <t xml:space="preserve">10/10 PASS is a verdict distribution, not accuracy - no oracle ran. Wilson 95%: zero failures in 10 still allows a true non-PASS rate up to 27.8% (B5 statistics.py). Batch 2 ran under policy 45c94e20 vs batch 1 4c52b4fb: upstream added Windows-only proxy env passthrough; macOS execution identical.</t>
+    <t xml:space="preserve">Verdict distribution, not accuracy - no oracle ran. 17/20 PASS; at n=20 with 3 non-PASS the observed non-PASS rate is 15%. Batches 2-3 ran under policy 45c94e20 vs batch 1 4c52b4fb (upstream Windows-only env passthrough; macOS identical).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$0.0000"/>
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="\$0.000"/>
     <numFmt numFmtId="168" formatCode="\$0.00"/>
-    <numFmt numFmtId="169" formatCode="0.0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -325,6 +450,22 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFD99100"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFE9425F"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="13"/>
       <color rgb="FF001928"/>
       <name val="Arial"/>
@@ -356,6 +497,29 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF001928"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FFD99100"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FFE9425F"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -425,7 +589,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -446,15 +610,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -462,27 +666,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -541,8 +725,8 @@
       <rgbColor rgb="FF00B88C"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FFD99100"/>
+      <rgbColor rgb="FFE9425F"/>
       <rgbColor rgb="FF646C76"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
@@ -796,7 +980,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -809,10 +993,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="10"/>
@@ -1431,6 +1615,566 @@
         <v>42</v>
       </c>
       <c r="R11" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>1597</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>5550</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>847207</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>51481</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0.217</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>9297</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q12" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>1541</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>4439</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>514280</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>25551</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>0.1263</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>9595</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1589</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>5294</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>767409</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>26127</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.1571</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>9740</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>1581</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>5341</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>751295</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>27279</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>9544</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>1557</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>4625</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>586377</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>22319</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>9247</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q16" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>1605</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>5437</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>880272</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>27882</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>0.1726</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>8542</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q17" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>1589</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>5780</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>796230</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>26568</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>0.1632</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>8224</v>
+      </c>
+      <c r="L18" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O18" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R18" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>1605</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>6035</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>873325</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>27452</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>0.174</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>8436</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q19" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R19" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>1597</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>5547</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>826863</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>27453</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>0.1669</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>8264</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O20" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q20" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R20" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>1557</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>4600</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>612566</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>25678</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>0.1372</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>8374</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P21" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q21" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R21" s="2" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1450,293 +2194,349 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
-        <v>53</v>
+      <c r="A1" s="7" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
+      <c r="A2" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="11" t="n">
+        <f aca="false">COUNTIF(Runs!L:L,"PASS")</f>
+        <v>17</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <f aca="false">AVERAGE(Runs!J2:J21)</f>
+        <v>71.95</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" s="11" t="n">
+        <f aca="false">COUNTIF(Runs!L:L,"FAIL")</f>
+        <v>1</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <f aca="false">AVERAGE(Runs!K2:K21)</f>
+        <v>9291.3</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="11" t="n">
+        <f aca="false">COUNTIF(Runs!L:L,"NEEDS_HUMAN")</f>
+        <v>2</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E8" s="13" t="n">
+        <f aca="false">AVERAGE(Runs!I2:I21)</f>
+        <v>0.16464</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="11" t="n">
+        <f aca="false">COUNTA(Runs!A:A)-1</f>
+        <v>20</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <f aca="false">SUM(Runs!I2:I21)</f>
+        <v>3.2928</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D10" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <f aca="false">AVERAGE(Runs!F2:F21)</f>
+        <v>5498.8</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="9" t="n">
-        <f aca="false">COUNTIF(Runs!L:L,"PASS")</f>
-        <v>10</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="10" t="n">
-        <f aca="false">AVERAGE(Runs!J2:J11)</f>
-        <v>75.4</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B8" s="9" t="n">
-        <f aca="false">COUNTIF(Runs!L:L,"FAIL")</f>
-        <v>0</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="10" t="n">
-        <f aca="false">AVERAGE(Runs!K2:K11)</f>
-        <v>9656.3</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B9" s="9" t="n">
-        <f aca="false">COUNTIF(Runs!L:L,"NEEDS_HUMAN")</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <f aca="false">AVERAGE(Runs!I2:I11)</f>
-        <v>0.16925</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="B10" s="9" t="n">
-        <f aca="false">COUNTA(Runs!A:A)-1</f>
-        <v>10</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="E10" s="12" t="n">
-        <f aca="false">SUM(Runs!I2:I11)</f>
-        <v>1.6925</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D11" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="E11" s="10" t="n">
-        <f aca="false">AVERAGE(Runs!F2:F11)</f>
-        <v>5732.8</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D12" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E12" s="13" t="n">
-        <f aca="false">AVERAGE(Runs!D2:D11)</f>
-        <v>21.5</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18" s="8" t="s">
+      <c r="D23" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C24" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B19" s="8" t="s">
+      <c r="D24" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="E24" s="18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B20" s="8" t="s">
+      <c r="C25" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C26" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="s">
-        <v>79</v>
+      <c r="D26" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
+      <c r="A28" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
+      <c r="A29" s="19"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="19" t="s">
+        <v>122</v>
+      </c>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="19"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="19"/>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A2:F4"/>
-    <mergeCell ref="A15:F16"/>
-    <mergeCell ref="A23:F25"/>
-    <mergeCell ref="A28:F30"/>
+  <mergeCells count="6">
+    <mergeCell ref="A2:F3"/>
+    <mergeCell ref="C13:F14"/>
+    <mergeCell ref="C15:F16"/>
+    <mergeCell ref="C17:F18"/>
+    <mergeCell ref="A28:F29"/>
+    <mergeCell ref="A32:F34"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>